<commit_message>
full files and codes
</commit_message>
<xml_diff>
--- a/Model_Predictions_vs_Actual.xlsx
+++ b/Model_Predictions_vs_Actual.xlsx
@@ -494,7 +494,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -514,7 +514,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -571,7 +571,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -597,7 +597,7 @@
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -685,7 +685,7 @@
         <v>1</v>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
         <v>2</v>
@@ -694,7 +694,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -754,7 +754,7 @@
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
@@ -848,7 +848,7 @@
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
@@ -871,7 +871,7 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
@@ -931,13 +931,13 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -954,7 +954,7 @@
         <v>2</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>2</v>
@@ -1105,7 +1105,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
         <v>2</v>
@@ -1131,10 +1131,10 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>2</v>
@@ -1148,7 +1148,7 @@
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1185,13 +1185,13 @@
         <v>1</v>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1211,7 +1211,7 @@
         <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -1225,19 +1225,19 @@
         <v>1</v>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
         <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1248,7 +1248,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1268,10 +1268,10 @@
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
         <v>1</v>
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -1308,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>2</v>
@@ -1334,7 +1334,7 @@
         <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1388,7 +1388,7 @@
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
         <v>2</v>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C50" t="n">
         <v>2</v>
@@ -1437,7 +1437,7 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -1531,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
         <v>1</v>
@@ -1608,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D59" t="n">
         <v>2</v>
@@ -1625,7 +1625,7 @@
         <v>0</v>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C60" t="n">
         <v>1</v>
@@ -1671,13 +1671,13 @@
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
         <v>2</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -1705,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="B64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
@@ -1765,7 +1765,7 @@
         <v>2</v>
       </c>
       <c r="B67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C67" t="n">
         <v>2</v>
@@ -1777,7 +1777,7 @@
         <v>2</v>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -1788,7 +1788,7 @@
         <v>2</v>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71" t="n">
         <v>1</v>
@@ -1894,7 +1894,7 @@
         <v>1</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F73" t="n">
         <v>2</v>
@@ -1908,7 +1908,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -1925,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C75" t="n">
         <v>1</v>
@@ -1968,7 +1968,7 @@
         <v>2</v>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -2017,7 +2017,7 @@
         <v>2</v>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -2117,7 +2117,7 @@
         <v>2</v>
       </c>
       <c r="F84" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -2145,13 +2145,13 @@
         <v>1</v>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C86" t="n">
         <v>2</v>
       </c>
       <c r="D86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86" t="n">
         <v>0</v>
@@ -2171,7 +2171,7 @@
         <v>2</v>
       </c>
       <c r="D87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" t="n">
         <v>0</v>
@@ -2185,16 +2185,16 @@
         <v>1</v>
       </c>
       <c r="B88" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C88" t="n">
         <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>1</v>
@@ -2211,7 +2211,7 @@
         <v>1</v>
       </c>
       <c r="D89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E89" t="n">
         <v>1</v>
@@ -2285,7 +2285,7 @@
         <v>1</v>
       </c>
       <c r="B93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C93" t="n">
         <v>1</v>
@@ -2331,7 +2331,7 @@
         <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E95" t="n">
         <v>1</v>
@@ -2408,7 +2408,7 @@
         <v>2</v>
       </c>
       <c r="C99" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2431,13 +2431,13 @@
         <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E100" t="n">
         <v>2</v>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -2445,13 +2445,13 @@
         <v>2</v>
       </c>
       <c r="B101" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C101" t="n">
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E101" t="n">
         <v>1</v>
@@ -2465,13 +2465,13 @@
         <v>0</v>
       </c>
       <c r="B102" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C102" t="n">
         <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E102" t="n">
         <v>2</v>
@@ -2531,10 +2531,10 @@
         <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F105" t="n">
         <v>2</v>
@@ -2691,7 +2691,7 @@
         <v>2</v>
       </c>
       <c r="D113" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E113" t="n">
         <v>2</v>
@@ -2745,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="B116" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" t="n">
         <v>1</v>
@@ -2831,7 +2831,7 @@
         <v>2</v>
       </c>
       <c r="D120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E120" t="n">
         <v>2</v>
@@ -2885,16 +2885,16 @@
         <v>0</v>
       </c>
       <c r="B123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F123" t="n">
         <v>2</v>
@@ -2928,7 +2928,7 @@
         <v>0</v>
       </c>
       <c r="C125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -2991,13 +2991,13 @@
         <v>1</v>
       </c>
       <c r="D128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -3005,13 +3005,13 @@
         <v>2</v>
       </c>
       <c r="B129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E129" t="n">
         <v>0</v>
@@ -3074,7 +3074,7 @@
         <v>1</v>
       </c>
       <c r="E132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F132" t="n">
         <v>1</v>
@@ -3105,7 +3105,7 @@
         <v>2</v>
       </c>
       <c r="B134" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C134" t="n">
         <v>2</v>
@@ -3165,7 +3165,7 @@
         <v>1</v>
       </c>
       <c r="B137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C137" t="n">
         <v>1</v>
@@ -3194,7 +3194,7 @@
         <v>2</v>
       </c>
       <c r="E138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F138" t="n">
         <v>2</v>
@@ -3211,10 +3211,10 @@
         <v>2</v>
       </c>
       <c r="D139" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F139" t="n">
         <v>2</v>
@@ -3225,19 +3225,19 @@
         <v>0</v>
       </c>
       <c r="B140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E140" t="n">
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141">
@@ -3251,7 +3251,7 @@
         <v>1</v>
       </c>
       <c r="D141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E141" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         <v>0</v>
       </c>
       <c r="B143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C143" t="n">
         <v>1</v>
@@ -3331,7 +3331,7 @@
         <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E145" t="n">
         <v>0</v>
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="B146" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C146" t="n">
         <v>2</v>
@@ -3371,7 +3371,7 @@
         <v>1</v>
       </c>
       <c r="D147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E147" t="n">
         <v>1</v>
@@ -3391,7 +3391,7 @@
         <v>2</v>
       </c>
       <c r="D148" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E148" t="n">
         <v>2</v>
@@ -3445,7 +3445,7 @@
         <v>1</v>
       </c>
       <c r="B151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C151" t="n">
         <v>1</v>
@@ -3465,7 +3465,7 @@
         <v>1</v>
       </c>
       <c r="B152" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C152" t="n">
         <v>1</v>
@@ -3477,7 +3477,7 @@
         <v>1</v>
       </c>
       <c r="F152" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153">
@@ -3491,13 +3491,13 @@
         <v>1</v>
       </c>
       <c r="D153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E153" t="n">
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -3514,7 +3514,7 @@
         <v>1</v>
       </c>
       <c r="E154" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F154" t="n">
         <v>2</v>
@@ -3571,10 +3571,10 @@
         <v>0</v>
       </c>
       <c r="D157" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E157" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F157" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
         <v>2</v>
       </c>
       <c r="E158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F158" t="n">
         <v>2</v>
@@ -3665,7 +3665,7 @@
         <v>0</v>
       </c>
       <c r="B162" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C162" t="n">
         <v>1</v>
@@ -3751,7 +3751,7 @@
         <v>1</v>
       </c>
       <c r="D166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E166" t="n">
         <v>1</v>
@@ -3771,7 +3771,7 @@
         <v>2</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E167" t="n">
         <v>2</v>
@@ -3788,10 +3788,10 @@
         <v>2</v>
       </c>
       <c r="C168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E168" t="n">
         <v>0</v>
@@ -3854,7 +3854,7 @@
         <v>2</v>
       </c>
       <c r="E171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F171" t="n">
         <v>2</v>
@@ -3888,7 +3888,7 @@
         <v>2</v>
       </c>
       <c r="C173" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D173" t="n">
         <v>2</v>
@@ -3925,7 +3925,7 @@
         <v>0</v>
       </c>
       <c r="B175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C175" t="n">
         <v>2</v>
@@ -3954,7 +3954,7 @@
         <v>1</v>
       </c>
       <c r="E176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F176" t="n">
         <v>1</v>
@@ -3991,7 +3991,7 @@
         <v>2</v>
       </c>
       <c r="D178" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E178" t="n">
         <v>0</v>
@@ -4005,16 +4005,16 @@
         <v>1</v>
       </c>
       <c r="B179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C179" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D179" t="n">
         <v>1</v>
       </c>
       <c r="E179" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F179" t="n">
         <v>2</v>
@@ -4065,7 +4065,7 @@
         <v>2</v>
       </c>
       <c r="B182" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C182" t="n">
         <v>2</v>
@@ -4085,7 +4085,7 @@
         <v>0</v>
       </c>
       <c r="B183" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C183" t="n">
         <v>1</v>
@@ -4094,7 +4094,7 @@
         <v>0</v>
       </c>
       <c r="E183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -4105,7 +4105,7 @@
         <v>1</v>
       </c>
       <c r="B184" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C184" t="n">
         <v>2</v>
@@ -4134,7 +4134,7 @@
         <v>2</v>
       </c>
       <c r="E185" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F185" t="n">
         <v>2</v>
@@ -4165,13 +4165,13 @@
         <v>2</v>
       </c>
       <c r="B187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C187" t="n">
         <v>1</v>
       </c>
       <c r="D187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E187" t="n">
         <v>2</v>
@@ -4188,10 +4188,10 @@
         <v>0</v>
       </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D188" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E188" t="n">
         <v>0</v>
@@ -4208,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="C189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D189" t="n">
         <v>0</v>
@@ -4231,10 +4231,10 @@
         <v>2</v>
       </c>
       <c r="D190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E190" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F190" t="n">
         <v>2</v>
@@ -4245,7 +4245,7 @@
         <v>1</v>
       </c>
       <c r="B191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C191" t="n">
         <v>1</v>
@@ -4271,7 +4271,7 @@
         <v>1</v>
       </c>
       <c r="D192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E192" t="n">
         <v>1</v>
@@ -4325,7 +4325,7 @@
         <v>0</v>
       </c>
       <c r="B195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C195" t="n">
         <v>1</v>
@@ -4354,7 +4354,7 @@
         <v>1</v>
       </c>
       <c r="E196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F196" t="n">
         <v>1</v>
@@ -4385,7 +4385,7 @@
         <v>0</v>
       </c>
       <c r="B198" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C198" t="n">
         <v>0</v>
@@ -4428,13 +4428,13 @@
         <v>1</v>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
       </c>
       <c r="E200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F200" t="n">
         <v>2</v>
@@ -4445,10 +4445,10 @@
         <v>1</v>
       </c>
       <c r="B201" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -4457,7 +4457,7 @@
         <v>2</v>
       </c>
       <c r="F201" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -4485,10 +4485,10 @@
         <v>0</v>
       </c>
       <c r="B203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D203" t="n">
         <v>2</v>
@@ -4528,13 +4528,13 @@
         <v>2</v>
       </c>
       <c r="C205" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D205" t="n">
         <v>0</v>
       </c>
       <c r="E205" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F205" t="n">
         <v>2</v>
@@ -4625,16 +4625,16 @@
         <v>0</v>
       </c>
       <c r="B210" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E210" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F210" t="n">
         <v>2</v>
@@ -4645,7 +4645,7 @@
         <v>1</v>
       </c>
       <c r="B211" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C211" t="n">
         <v>1</v>
@@ -4685,7 +4685,7 @@
         <v>2</v>
       </c>
       <c r="B213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C213" t="n">
         <v>1</v>
@@ -4708,10 +4708,10 @@
         <v>0</v>
       </c>
       <c r="C214" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D214" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E214" t="n">
         <v>0</v>
@@ -4748,7 +4748,7 @@
         <v>2</v>
       </c>
       <c r="C216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -4771,10 +4771,10 @@
         <v>1</v>
       </c>
       <c r="D217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E217" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F217" t="n">
         <v>1</v>
@@ -4785,7 +4785,7 @@
         <v>2</v>
       </c>
       <c r="B218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C218" t="n">
         <v>1</v>
@@ -4794,10 +4794,10 @@
         <v>0</v>
       </c>
       <c r="E218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="219">
@@ -4805,10 +4805,10 @@
         <v>2</v>
       </c>
       <c r="B219" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C219" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D219" t="n">
         <v>0</v>
@@ -4825,7 +4825,7 @@
         <v>1</v>
       </c>
       <c r="B220" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C220" t="n">
         <v>2</v>
@@ -4854,7 +4854,7 @@
         <v>2</v>
       </c>
       <c r="E221" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -4974,7 +4974,7 @@
         <v>2</v>
       </c>
       <c r="E227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F227" t="n">
         <v>2</v>
@@ -5151,13 +5151,13 @@
         <v>1</v>
       </c>
       <c r="D236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E236" t="n">
         <v>1</v>
       </c>
       <c r="F236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">
@@ -5191,7 +5191,7 @@
         <v>1</v>
       </c>
       <c r="D238" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E238" t="n">
         <v>0</v>
@@ -5214,7 +5214,7 @@
         <v>2</v>
       </c>
       <c r="E239" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F239" t="n">
         <v>2</v>

</xml_diff>